<commit_message>
Update data sources and add code to look at forecasts vs post-season for Fraser pink and sockeye
</commit_message>
<xml_diff>
--- a/data/data-sources_2025.xlsx
+++ b/data/data-sources_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephaniepeacock/Library/CloudStorage/Dropbox-SalmonWatersheds/Stephanie Peacock/X Drive/1_PROJECTS/1_Active/State of Salmon/2_Data &amp; Analysis/state-of-salmon/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0040D675-0E64-FD4C-BE0E-44821F354C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B45AE43-5A0C-D349-9474-1DDE45AF61D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9860" yWindow="4160" windowWidth="26840" windowHeight="13780" xr2:uid="{E96813F5-1777-F041-8F52-E9C9A952FEDD}"/>
+    <workbookView xWindow="9840" yWindow="4160" windowWidth="26840" windowHeight="13780" xr2:uid="{E96813F5-1777-F041-8F52-E9C9A952FEDD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated data and output to reflect (1) new total abundance for Fraser Chinook from Chuck Parken and (2) updated Okanagan sockeye from Ogden et al. (2025)
</commit_message>
<xml_diff>
--- a/data/data-sources_2025.xlsx
+++ b/data/data-sources_2025.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephaniepeacock/Library/CloudStorage/Dropbox-SalmonWatersheds/Stephanie Peacock/X Drive/1_PROJECTS/1_Active/State of Salmon/2_Data &amp; Analysis/state-of-salmon/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B45AE43-5A0C-D349-9474-1DDE45AF61D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A57CE39F-F4BA-374F-982F-9C54C7631D30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9840" yWindow="4160" windowWidth="26840" windowHeight="13780" xr2:uid="{E96813F5-1777-F041-8F52-E9C9A952FEDD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>source_id</t>
   </si>
@@ -194,12 +194,47 @@
   <si>
     <t>OBMEP. 2025. 2024 Okanogan Subbasin Steelhead Spawning Abundance and Distribution. Colville Confederated Tribes Fish and Wildlife Department, Nespelem, WA. Report submitted to the Bonneville Power Administration, Project No. 2003-022-00. Available at https://www.okanoganmonitoring.org/ [accessed Mar 18, 2025].</t>
   </si>
+  <si>
+    <t>Ogden_20250901</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Ogden, A.D., Alex, K., Pestal, G., Alameddine, I., Davis, B., Judson, B., Stiff, H., and Pham, S. 2025. Wild Salmon Policy Status, Limit Reference Point, and Candidate Escapement Goals for Okanagan Sockeye Salmon. Canadian Science Advisory Secretariat Research Document </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2025/046</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: xii + 102 p. Available from https://waves-vagues.dfo-mpo.gc.ca/library-bibliotheque/41302795.pdf</t>
+    </r>
+  </si>
+  <si>
+    <t>Parken_20251023</t>
+  </si>
+  <si>
+    <t>Parken, Chuck. 2025. Fraser Chinook escapement and terminal run by Stock Managenent Unit, 1979 - 2024. Provided to Pacific Salmon Foundation by Chuck Parken (DFO) on October 23, 2025.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -224,6 +259,14 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -595,7 +638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24029AEC-6FE5-6340-8374-FCF69BAFD37B}">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" customWidth="1"/>
@@ -786,6 +829,22 @@
         <v>45</v>
       </c>
     </row>
+    <row r="24" spans="1:2" ht="51" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>